<commit_message>
Excel verilerini güncelle (yeni güncelleme)
</commit_message>
<xml_diff>
--- a/25-26-Bahar-Final-OİS.xlsx
+++ b/25-26-Bahar-Final-OİS.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EF7BC76-E170-4616-871F-4BD4D0B13657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{016EB8B8-7FB3-42B9-908A-19110CFECB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1192,6 +1192,9 @@
     <t>Dr. Öğr. Üyesi Cevahir Parlak</t>
   </si>
   <si>
+    <t>Arş. Gör. Berke Erdoğan</t>
+  </si>
+  <si>
     <t>Doç.Dr. Nihan Akıncılar Köseoğlu</t>
   </si>
   <si>
@@ -1232,9 +1235,6 @@
   </si>
   <si>
     <t>Dr.Öğr.Üyesi Tuğba Baş</t>
-  </si>
-  <si>
-    <t>Arş. Gör. Berke Erdoğan</t>
   </si>
   <si>
     <t>INTF202</t>
@@ -18542,10 +18542,10 @@
         <v>384</v>
       </c>
       <c r="I477" s="294" t="s">
-        <v>315</v>
+        <v>385</v>
       </c>
       <c r="J477" s="294" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="478" spans="1:10" ht="15.75">
@@ -18577,12 +18577,12 @@
         <v>263</v>
       </c>
       <c r="J478" s="294" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="479" spans="1:10" ht="15.75">
       <c r="A479" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B479">
         <v>1</v>
@@ -18618,14 +18618,14 @@
     </row>
     <row r="481" spans="1:10" ht="15.75">
       <c r="A481" s="293" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="H481" s="294"/>
       <c r="I481" s="294"/>
     </row>
     <row r="482" spans="1:10" ht="15.75">
       <c r="A482" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B482">
         <v>1</v>
@@ -18657,7 +18657,7 @@
     </row>
     <row r="483" spans="1:10" ht="15.75">
       <c r="A483" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B483">
         <v>1</v>
@@ -18686,7 +18686,7 @@
     </row>
     <row r="484" spans="1:10" ht="15.75">
       <c r="A484" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B484">
         <v>1</v>
@@ -18718,7 +18718,7 @@
     </row>
     <row r="485" spans="1:10" ht="15.75">
       <c r="A485" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B485">
         <v>1</v>
@@ -18727,7 +18727,7 @@
         <v>244</v>
       </c>
       <c r="D485" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E485" s="275">
         <v>46202</v>
@@ -18739,7 +18739,7 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="H485" s="294" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="I485" s="294" t="s">
         <v>315</v>
@@ -18747,7 +18747,7 @@
     </row>
     <row r="486" spans="1:10" ht="15.75">
       <c r="A486" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B486">
         <v>1</v>
@@ -18776,7 +18776,7 @@
     </row>
     <row r="488" spans="1:10">
       <c r="A488" s="329" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B488" s="330"/>
       <c r="C488" s="330"/>
@@ -18790,7 +18790,7 @@
     </row>
     <row r="489" spans="1:10" s="328" customFormat="1" ht="15.75">
       <c r="A489" s="331" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B489" s="331">
         <v>1</v>
@@ -18811,10 +18811,10 @@
         <v>0.4375</v>
       </c>
       <c r="H489" s="334" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I489" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J489" s="331"/>
     </row>
@@ -18841,10 +18841,10 @@
         <v>0.4375</v>
       </c>
       <c r="H490" s="334" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I490" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J490" s="331" t="s">
         <v>401</v>
@@ -18876,10 +18876,10 @@
         <v>403</v>
       </c>
       <c r="I491" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J491" s="335" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="492" spans="1:10" s="328" customFormat="1" ht="15.75">
@@ -18908,7 +18908,7 @@
         <v>406</v>
       </c>
       <c r="I492" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J492" s="353" t="s">
         <v>407</v>
@@ -18940,7 +18940,7 @@
         <v>409</v>
       </c>
       <c r="I493" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J493" s="336"/>
     </row>
@@ -18970,7 +18970,7 @@
         <v>412</v>
       </c>
       <c r="I494" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J494" s="336" t="s">
         <v>315</v>
@@ -18999,10 +18999,10 @@
         <v>0.4375</v>
       </c>
       <c r="H495" s="334" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I495" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J495" s="336" t="s">
         <v>317</v>
@@ -19064,7 +19064,7 @@
         <v>412</v>
       </c>
       <c r="I497" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J497" s="336"/>
     </row>
@@ -19094,7 +19094,7 @@
         <v>412</v>
       </c>
       <c r="I498" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J498" s="336"/>
     </row>
@@ -19124,7 +19124,7 @@
         <v>409</v>
       </c>
       <c r="I499" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J499" s="336"/>
     </row>
@@ -19151,7 +19151,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="H500" s="334" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I500" s="335" t="s">
         <v>409</v>
@@ -19184,10 +19184,10 @@
         <v>421</v>
       </c>
       <c r="I501" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J501" s="336" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="502" spans="1:10" s="328" customFormat="1" ht="15.75">
@@ -19216,7 +19216,7 @@
         <v>423</v>
       </c>
       <c r="I502" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J502" s="336"/>
     </row>
@@ -19246,7 +19246,7 @@
         <v>423</v>
       </c>
       <c r="I503" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J503" s="336"/>
     </row>
@@ -19276,7 +19276,7 @@
         <v>412</v>
       </c>
       <c r="I504" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J504" s="336"/>
     </row>
@@ -19336,7 +19336,7 @@
         <v>423</v>
       </c>
       <c r="I506" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J506" s="336"/>
     </row>
@@ -19366,7 +19366,7 @@
         <v>421</v>
       </c>
       <c r="I507" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J507" s="336"/>
     </row>
@@ -19396,7 +19396,7 @@
         <v>412</v>
       </c>
       <c r="I508" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J508" s="336" t="s">
         <v>366</v>
@@ -19428,7 +19428,7 @@
         <v>432</v>
       </c>
       <c r="I509" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J509" s="336"/>
     </row>
@@ -19458,7 +19458,7 @@
         <v>432</v>
       </c>
       <c r="I510" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J510" s="336"/>
     </row>
@@ -19488,7 +19488,7 @@
         <v>432</v>
       </c>
       <c r="I511" s="335" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="J511" s="336"/>
     </row>
@@ -19561,7 +19561,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="H515" s="307" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I515" s="307" t="s">
         <v>409</v>
@@ -22873,17 +22873,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="46f9de43-f693-4abd-b3da-16a9446d5b24" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="123f497b-f32e-4e02-92f3-8b4fa7417143">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -22892,7 +22881,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Belge" ma:contentTypeID="0x010100256068D72C9EFB48AF3F54B18B894F64" ma:contentTypeVersion="10" ma:contentTypeDescription="Yeni belge oluşturun." ma:contentTypeScope="" ma:versionID="43cc1ef052e03bb8a5b634da50b07d31">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="123f497b-f32e-4e02-92f3-8b4fa7417143" xmlns:ns3="46f9de43-f693-4abd-b3da-16a9446d5b24" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0a3b51fdaec3d0484dcb0692a12b6b92" ns2:_="" ns3:_="">
     <xsd:import namespace="123f497b-f32e-4e02-92f3-8b4fa7417143"/>
@@ -23081,14 +23070,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="46f9de43-f693-4abd-b3da-16a9446d5b24" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="123f497b-f32e-4e02-92f3-8b4fa7417143">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A88D52BA-A6DF-483C-98B0-475005FD20A6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B11B433E-0496-41C4-9F25-23499B75A235}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B11B433E-0496-41C4-9F25-23499B75A235}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FDAEC64-9782-4808-ADE6-A4491D0F9D2C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FDAEC64-9782-4808-ADE6-A4491D0F9D2C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A88D52BA-A6DF-483C-98B0-475005FD20A6}"/>
 </file>
</xml_diff>